<commit_message>
Add a function to create a link to the report.
</commit_message>
<xml_diff>
--- a/templete/templete.WTS.xlsx
+++ b/templete/templete.WTS.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mioka\AppData\Local\Temp\scp18923\data1\labTools\worksheet\version\v3.0.0\templete\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mioka\AppData\Local\Temp\scp38216\data1\labTools\worksheet\version\v3.1.0\templete\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC514379-15EE-44BB-8F11-C3C7D569421B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6699B01D-1237-4574-8367-FED7972A51DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-75" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21555" yWindow="2550" windowWidth="21075" windowHeight="12825" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="work_sheet" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">work_sheet!$A$1:$T$55</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">work_sheet!$A$1:$T$54</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="54">
   <si>
     <t>run_id</t>
   </si>
@@ -232,16 +232,6 @@
   </si>
   <si>
     <t>)            WET(</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>レポートに文字化けがないか確認する</t>
-    <rPh sb="5" eb="8">
-      <t>モジバ</t>
-    </rPh>
-    <rPh sb="13" eb="15">
-      <t>カクニン</t>
-    </rPh>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -449,13 +439,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>パイプラインで生成されたレポートをプリントアウトする（2in1,白黒両面印刷）</t>
-    <rPh sb="7" eb="9">
-      <t>セイセイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>OncoStationで SendMail ⇒ Upload Report ボタンを押下する</t>
     <rPh sb="42" eb="44">
       <t>オウカ</t>
@@ -532,6 +515,10 @@
     <rPh sb="39" eb="41">
       <t>ツイカ</t>
     </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>レポートをプリントアウトする（2in1,白黒両面印刷）</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -1330,7 +1317,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:T55"/>
+  <dimension ref="B1:T54"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="8.625" customWidth="1"/>
@@ -1350,7 +1337,7 @@
   <sheetData>
     <row r="1" spans="2:20" x14ac:dyDescent="0.4">
       <c r="B1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="2:20" x14ac:dyDescent="0.4">
@@ -1381,7 +1368,7 @@
       </c>
       <c r="Q2" s="43"/>
       <c r="R2" s="37" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="S2" s="37"/>
       <c r="T2" s="37"/>
@@ -1551,7 +1538,7 @@
         <v>1</v>
       </c>
       <c r="C11" s="52" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D11" s="53"/>
       <c r="E11" s="53"/>
@@ -1578,7 +1565,7 @@
         <v>2</v>
       </c>
       <c r="C12" s="52" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D12" s="53"/>
       <c r="E12" s="53"/>
@@ -1605,7 +1592,7 @@
         <v>3</v>
       </c>
       <c r="C13" s="52" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D13" s="53"/>
       <c r="E13" s="53"/>
@@ -1659,7 +1646,7 @@
         <v>5</v>
       </c>
       <c r="C15" s="52" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D15" s="53"/>
       <c r="E15" s="53"/>
@@ -1684,7 +1671,7 @@
     <row r="16" spans="2:20" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B16" s="16"/>
       <c r="C16" s="27" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D16" s="28"/>
       <c r="E16" s="28"/>
@@ -1694,18 +1681,18 @@
       <c r="I16" s="28"/>
       <c r="J16" s="29"/>
       <c r="K16" s="27" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L16" s="28"/>
       <c r="M16" s="28"/>
       <c r="N16" s="28"/>
       <c r="O16" s="28"/>
       <c r="P16" s="30" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Q16" s="30"/>
       <c r="R16" s="13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="S16" s="23"/>
       <c r="T16" s="24"/>
@@ -1713,22 +1700,22 @@
     <row r="17" spans="2:20" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B17" s="16"/>
       <c r="C17" s="33" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D17" s="33"/>
       <c r="E17" s="33"/>
       <c r="F17" s="34" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G17" s="35"/>
       <c r="H17" s="35"/>
       <c r="I17" s="35"/>
       <c r="J17" s="36"/>
       <c r="K17" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="L17" s="34" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="M17" s="35"/>
       <c r="N17" s="35"/>
@@ -1746,22 +1733,22 @@
     <row r="18" spans="2:20" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B18" s="16"/>
       <c r="C18" s="33" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D18" s="33"/>
       <c r="E18" s="33"/>
       <c r="F18" s="34" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G18" s="35"/>
       <c r="H18" s="35"/>
       <c r="I18" s="35"/>
       <c r="J18" s="36"/>
       <c r="K18" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="L18" s="34" t="s">
         <v>49</v>
-      </c>
-      <c r="L18" s="34" t="s">
-        <v>51</v>
       </c>
       <c r="M18" s="35"/>
       <c r="N18" s="35"/>
@@ -1776,203 +1763,199 @@
       <c r="S18" s="23"/>
       <c r="T18" s="24"/>
     </row>
-    <row r="19" spans="2:20" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:20" x14ac:dyDescent="0.4">
       <c r="B19" s="2">
         <v>6</v>
       </c>
-      <c r="C19" s="75" t="s">
-        <v>41</v>
-      </c>
-      <c r="D19" s="76"/>
-      <c r="E19" s="76"/>
-      <c r="F19" s="76"/>
-      <c r="G19" s="76"/>
-      <c r="H19" s="76"/>
-      <c r="I19" s="76"/>
-      <c r="J19" s="76"/>
-      <c r="K19" s="76"/>
-      <c r="L19" s="76"/>
-      <c r="M19" s="76"/>
-      <c r="N19" s="76"/>
-      <c r="O19" s="76"/>
-      <c r="P19" s="76"/>
-      <c r="Q19" s="76"/>
-      <c r="R19" s="77"/>
+      <c r="C19" s="60" t="s">
+        <v>35</v>
+      </c>
+      <c r="D19" s="60"/>
+      <c r="E19" s="60"/>
+      <c r="F19" s="60"/>
+      <c r="G19" s="60"/>
+      <c r="H19" s="60"/>
+      <c r="I19" s="60"/>
+      <c r="J19" s="60"/>
+      <c r="K19" s="60"/>
+      <c r="L19" s="60"/>
+      <c r="M19" s="60"/>
+      <c r="N19" s="60"/>
+      <c r="O19" s="60"/>
+      <c r="P19" s="60"/>
+      <c r="Q19" s="60"/>
+      <c r="R19" s="60"/>
       <c r="S19" s="34" t="s">
         <v>9</v>
       </c>
       <c r="T19" s="36"/>
     </row>
-    <row r="20" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B20" s="2">
+    <row r="20" spans="2:20" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B20" s="15">
         <v>7</v>
       </c>
-      <c r="C20" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="D20" s="53"/>
-      <c r="E20" s="53"/>
-      <c r="F20" s="53"/>
-      <c r="G20" s="53"/>
-      <c r="H20" s="53"/>
-      <c r="I20" s="53"/>
-      <c r="J20" s="53"/>
-      <c r="K20" s="53"/>
-      <c r="L20" s="53"/>
-      <c r="M20" s="53"/>
-      <c r="N20" s="53"/>
-      <c r="O20" s="53"/>
-      <c r="P20" s="53"/>
-      <c r="Q20" s="53"/>
-      <c r="R20" s="54"/>
-      <c r="S20" s="3" t="s">
+      <c r="C20" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="19"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="19"/>
+      <c r="J20" s="19"/>
+      <c r="K20" s="19"/>
+      <c r="L20" s="19"/>
+      <c r="M20" s="19"/>
+      <c r="N20" s="19"/>
+      <c r="O20" s="19"/>
+      <c r="P20" s="19"/>
+      <c r="Q20" s="19"/>
+      <c r="R20" s="20"/>
+      <c r="S20" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="T20" s="3" t="s">
+      <c r="T20" s="22"/>
+    </row>
+    <row r="21" spans="2:20" x14ac:dyDescent="0.4">
+      <c r="B21" s="16"/>
+      <c r="C21" s="45" t="s">
+        <v>36</v>
+      </c>
+      <c r="D21" s="46"/>
+      <c r="E21" s="46"/>
+      <c r="F21" s="46"/>
+      <c r="G21" s="46"/>
+      <c r="H21" s="46"/>
+      <c r="I21" s="46"/>
+      <c r="J21" s="46"/>
+      <c r="K21" s="46"/>
+      <c r="L21" s="46"/>
+      <c r="M21" s="46"/>
+      <c r="N21" s="46"/>
+      <c r="O21" s="46"/>
+      <c r="P21" s="46"/>
+      <c r="Q21" s="46"/>
+      <c r="R21" s="47"/>
+      <c r="S21" s="23"/>
+      <c r="T21" s="24"/>
+    </row>
+    <row r="22" spans="2:20" x14ac:dyDescent="0.4">
+      <c r="B22" s="17"/>
+      <c r="C22" s="74" t="s">
+        <v>25</v>
+      </c>
+      <c r="D22" s="70"/>
+      <c r="E22" s="70"/>
+      <c r="F22" s="70"/>
+      <c r="G22" s="70"/>
+      <c r="H22" s="70"/>
+      <c r="I22" s="70"/>
+      <c r="J22" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="K22" s="11"/>
+      <c r="L22" s="11"/>
+      <c r="M22" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="N22" s="70"/>
+      <c r="O22" s="70"/>
+      <c r="P22" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q22" s="9"/>
+      <c r="R22" s="6"/>
+      <c r="S22" s="25"/>
+      <c r="T22" s="26"/>
+    </row>
+    <row r="23" spans="2:20" x14ac:dyDescent="0.4">
+      <c r="B23" s="2">
+        <v>8</v>
+      </c>
+      <c r="C23" s="52" t="s">
+        <v>8</v>
+      </c>
+      <c r="D23" s="53"/>
+      <c r="E23" s="53"/>
+      <c r="F23" s="53"/>
+      <c r="G23" s="53"/>
+      <c r="H23" s="53"/>
+      <c r="I23" s="53"/>
+      <c r="J23" s="53"/>
+      <c r="K23" s="53"/>
+      <c r="L23" s="53"/>
+      <c r="M23" s="53"/>
+      <c r="N23" s="53"/>
+      <c r="O23" s="53"/>
+      <c r="P23" s="53"/>
+      <c r="Q23" s="53"/>
+      <c r="R23" s="54"/>
+      <c r="S23" s="34" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="21" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B21" s="2">
-        <v>8</v>
-      </c>
-      <c r="C21" s="52" t="s">
-        <v>8</v>
-      </c>
-      <c r="D21" s="53"/>
-      <c r="E21" s="53"/>
-      <c r="F21" s="53"/>
-      <c r="G21" s="53"/>
-      <c r="H21" s="53"/>
-      <c r="I21" s="53"/>
-      <c r="J21" s="53"/>
-      <c r="K21" s="53"/>
-      <c r="L21" s="53"/>
-      <c r="M21" s="53"/>
-      <c r="N21" s="53"/>
-      <c r="O21" s="53"/>
-      <c r="P21" s="53"/>
-      <c r="Q21" s="53"/>
-      <c r="R21" s="54"/>
-      <c r="S21" s="3" t="s">
+      <c r="T23" s="36"/>
+    </row>
+    <row r="24" spans="2:20" x14ac:dyDescent="0.4">
+      <c r="B24" s="2">
         <v>9</v>
       </c>
-      <c r="T21" s="3" t="s">
+      <c r="C24" s="38" t="s">
+        <v>40</v>
+      </c>
+      <c r="D24" s="39"/>
+      <c r="E24" s="39"/>
+      <c r="F24" s="39"/>
+      <c r="G24" s="39"/>
+      <c r="H24" s="39"/>
+      <c r="I24" s="39"/>
+      <c r="J24" s="39"/>
+      <c r="K24" s="39"/>
+      <c r="L24" s="39"/>
+      <c r="M24" s="39"/>
+      <c r="N24" s="39"/>
+      <c r="O24" s="39"/>
+      <c r="P24" s="39"/>
+      <c r="Q24" s="39"/>
+      <c r="R24" s="40"/>
+      <c r="S24" s="34" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="22" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B22" s="2">
+      <c r="T24" s="36"/>
+    </row>
+    <row r="25" spans="2:20" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B25" s="2">
+        <v>10</v>
+      </c>
+      <c r="C25" s="75" t="s">
+        <v>53</v>
+      </c>
+      <c r="D25" s="76"/>
+      <c r="E25" s="76"/>
+      <c r="F25" s="76"/>
+      <c r="G25" s="76"/>
+      <c r="H25" s="76"/>
+      <c r="I25" s="76"/>
+      <c r="J25" s="76"/>
+      <c r="K25" s="76"/>
+      <c r="L25" s="76"/>
+      <c r="M25" s="76"/>
+      <c r="N25" s="76"/>
+      <c r="O25" s="76"/>
+      <c r="P25" s="76"/>
+      <c r="Q25" s="76"/>
+      <c r="R25" s="77"/>
+      <c r="S25" s="34" t="s">
         <v>9</v>
       </c>
-      <c r="C22" s="60" t="s">
-        <v>36</v>
-      </c>
-      <c r="D22" s="60"/>
-      <c r="E22" s="60"/>
-      <c r="F22" s="60"/>
-      <c r="G22" s="60"/>
-      <c r="H22" s="60"/>
-      <c r="I22" s="60"/>
-      <c r="J22" s="60"/>
-      <c r="K22" s="60"/>
-      <c r="L22" s="60"/>
-      <c r="M22" s="60"/>
-      <c r="N22" s="60"/>
-      <c r="O22" s="60"/>
-      <c r="P22" s="60"/>
-      <c r="Q22" s="60"/>
-      <c r="R22" s="60"/>
-      <c r="S22" s="34" t="s">
-        <v>9</v>
-      </c>
-      <c r="T22" s="36"/>
-    </row>
-    <row r="23" spans="2:20" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B23" s="15">
-        <v>10</v>
-      </c>
-      <c r="C23" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="D23" s="19"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="19"/>
-      <c r="G23" s="19"/>
-      <c r="H23" s="19"/>
-      <c r="I23" s="19"/>
-      <c r="J23" s="19"/>
-      <c r="K23" s="19"/>
-      <c r="L23" s="19"/>
-      <c r="M23" s="19"/>
-      <c r="N23" s="19"/>
-      <c r="O23" s="19"/>
-      <c r="P23" s="19"/>
-      <c r="Q23" s="19"/>
-      <c r="R23" s="20"/>
-      <c r="S23" s="21" t="s">
-        <v>9</v>
-      </c>
-      <c r="T23" s="22"/>
-    </row>
-    <row r="24" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B24" s="16"/>
-      <c r="C24" s="45" t="s">
-        <v>37</v>
-      </c>
-      <c r="D24" s="46"/>
-      <c r="E24" s="46"/>
-      <c r="F24" s="46"/>
-      <c r="G24" s="46"/>
-      <c r="H24" s="46"/>
-      <c r="I24" s="46"/>
-      <c r="J24" s="46"/>
-      <c r="K24" s="46"/>
-      <c r="L24" s="46"/>
-      <c r="M24" s="46"/>
-      <c r="N24" s="46"/>
-      <c r="O24" s="46"/>
-      <c r="P24" s="46"/>
-      <c r="Q24" s="46"/>
-      <c r="R24" s="47"/>
-      <c r="S24" s="23"/>
-      <c r="T24" s="24"/>
-    </row>
-    <row r="25" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B25" s="17"/>
-      <c r="C25" s="74" t="s">
-        <v>25</v>
-      </c>
-      <c r="D25" s="70"/>
-      <c r="E25" s="70"/>
-      <c r="F25" s="70"/>
-      <c r="G25" s="70"/>
-      <c r="H25" s="70"/>
-      <c r="I25" s="70"/>
-      <c r="J25" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="K25" s="11"/>
-      <c r="L25" s="11"/>
-      <c r="M25" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="N25" s="70"/>
-      <c r="O25" s="70"/>
-      <c r="P25" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q25" s="9"/>
-      <c r="R25" s="6"/>
-      <c r="S25" s="25"/>
-      <c r="T25" s="26"/>
+      <c r="T25" s="36"/>
     </row>
     <row r="26" spans="2:20" x14ac:dyDescent="0.4">
       <c r="B26" s="2">
         <v>11</v>
       </c>
       <c r="C26" s="38" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="D26" s="39"/>
       <c r="E26" s="39"/>
@@ -1999,7 +1982,7 @@
         <v>12</v>
       </c>
       <c r="C27" s="38" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="D27" s="39"/>
       <c r="E27" s="39"/>
@@ -2022,75 +2005,69 @@
       <c r="T27" s="36"/>
     </row>
     <row r="28" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B28" s="2">
-        <v>13</v>
-      </c>
-      <c r="C28" s="38" t="s">
-        <v>14</v>
-      </c>
-      <c r="D28" s="39"/>
-      <c r="E28" s="39"/>
-      <c r="F28" s="39"/>
-      <c r="G28" s="39"/>
-      <c r="H28" s="39"/>
-      <c r="I28" s="39"/>
-      <c r="J28" s="39"/>
-      <c r="K28" s="39"/>
-      <c r="L28" s="39"/>
-      <c r="M28" s="39"/>
-      <c r="N28" s="39"/>
-      <c r="O28" s="39"/>
-      <c r="P28" s="39"/>
-      <c r="Q28" s="39"/>
-      <c r="R28" s="40"/>
-      <c r="S28" s="34" t="s">
-        <v>9</v>
-      </c>
-      <c r="T28" s="36"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="7"/>
+      <c r="D28" s="7"/>
+      <c r="E28" s="7"/>
+      <c r="F28" s="7"/>
+      <c r="G28" s="7"/>
+      <c r="H28" s="7"/>
+      <c r="I28" s="7"/>
+      <c r="J28" s="7"/>
+      <c r="K28" s="7"/>
+      <c r="L28" s="7"/>
+      <c r="M28" s="7"/>
+      <c r="N28" s="7"/>
+      <c r="O28" s="7"/>
+      <c r="P28" s="7"/>
+      <c r="Q28" s="7"/>
+      <c r="R28" s="8"/>
+      <c r="S28" s="8"/>
+      <c r="T28" s="8"/>
     </row>
     <row r="29" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B29" s="4"/>
-      <c r="C29" s="7"/>
-      <c r="D29" s="7"/>
-      <c r="E29" s="7"/>
-      <c r="F29" s="7"/>
-      <c r="G29" s="7"/>
-      <c r="H29" s="7"/>
-      <c r="I29" s="7"/>
-      <c r="J29" s="7"/>
-      <c r="K29" s="7"/>
-      <c r="L29" s="7"/>
-      <c r="M29" s="7"/>
-      <c r="N29" s="7"/>
-      <c r="O29" s="7"/>
-      <c r="P29" s="7"/>
-      <c r="Q29" s="7"/>
-      <c r="R29" s="8"/>
-      <c r="S29" s="8"/>
-      <c r="T29" s="8"/>
+      <c r="B29" s="61" t="s">
+        <v>21</v>
+      </c>
+      <c r="C29" s="62"/>
+      <c r="D29" s="62"/>
+      <c r="E29" s="62"/>
+      <c r="F29" s="62"/>
+      <c r="G29" s="62"/>
+      <c r="H29" s="62"/>
+      <c r="I29" s="62"/>
+      <c r="J29" s="62"/>
+      <c r="K29" s="62"/>
+      <c r="L29" s="62"/>
+      <c r="M29" s="62"/>
+      <c r="N29" s="62"/>
+      <c r="O29" s="62"/>
+      <c r="P29" s="62"/>
+      <c r="Q29" s="62"/>
+      <c r="R29" s="62"/>
+      <c r="S29" s="62"/>
+      <c r="T29" s="63"/>
     </row>
     <row r="30" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B30" s="61" t="s">
-        <v>21</v>
-      </c>
-      <c r="C30" s="62"/>
-      <c r="D30" s="62"/>
-      <c r="E30" s="62"/>
-      <c r="F30" s="62"/>
-      <c r="G30" s="62"/>
-      <c r="H30" s="62"/>
-      <c r="I30" s="62"/>
-      <c r="J30" s="62"/>
-      <c r="K30" s="62"/>
-      <c r="L30" s="62"/>
-      <c r="M30" s="62"/>
-      <c r="N30" s="62"/>
-      <c r="O30" s="62"/>
-      <c r="P30" s="62"/>
-      <c r="Q30" s="62"/>
-      <c r="R30" s="62"/>
-      <c r="S30" s="62"/>
-      <c r="T30" s="63"/>
+      <c r="B30" s="64"/>
+      <c r="C30" s="65"/>
+      <c r="D30" s="65"/>
+      <c r="E30" s="65"/>
+      <c r="F30" s="65"/>
+      <c r="G30" s="65"/>
+      <c r="H30" s="65"/>
+      <c r="I30" s="65"/>
+      <c r="J30" s="65"/>
+      <c r="K30" s="65"/>
+      <c r="L30" s="65"/>
+      <c r="M30" s="65"/>
+      <c r="N30" s="65"/>
+      <c r="O30" s="65"/>
+      <c r="P30" s="65"/>
+      <c r="Q30" s="65"/>
+      <c r="R30" s="65"/>
+      <c r="S30" s="65"/>
+      <c r="T30" s="66"/>
     </row>
     <row r="31" spans="2:20" x14ac:dyDescent="0.4">
       <c r="B31" s="64"/>
@@ -2135,69 +2112,69 @@
       <c r="T32" s="66"/>
     </row>
     <row r="33" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B33" s="64"/>
-      <c r="C33" s="65"/>
-      <c r="D33" s="65"/>
-      <c r="E33" s="65"/>
-      <c r="F33" s="65"/>
-      <c r="G33" s="65"/>
-      <c r="H33" s="65"/>
-      <c r="I33" s="65"/>
-      <c r="J33" s="65"/>
-      <c r="K33" s="65"/>
-      <c r="L33" s="65"/>
-      <c r="M33" s="65"/>
-      <c r="N33" s="65"/>
-      <c r="O33" s="65"/>
-      <c r="P33" s="65"/>
-      <c r="Q33" s="65"/>
-      <c r="R33" s="65"/>
-      <c r="S33" s="65"/>
-      <c r="T33" s="66"/>
+      <c r="B33" s="67"/>
+      <c r="C33" s="68"/>
+      <c r="D33" s="68"/>
+      <c r="E33" s="68"/>
+      <c r="F33" s="68"/>
+      <c r="G33" s="68"/>
+      <c r="H33" s="68"/>
+      <c r="I33" s="68"/>
+      <c r="J33" s="68"/>
+      <c r="K33" s="68"/>
+      <c r="L33" s="68"/>
+      <c r="M33" s="68"/>
+      <c r="N33" s="68"/>
+      <c r="O33" s="68"/>
+      <c r="P33" s="68"/>
+      <c r="Q33" s="68"/>
+      <c r="R33" s="68"/>
+      <c r="S33" s="68"/>
+      <c r="T33" s="69"/>
     </row>
     <row r="34" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B34" s="67"/>
-      <c r="C34" s="68"/>
-      <c r="D34" s="68"/>
-      <c r="E34" s="68"/>
-      <c r="F34" s="68"/>
-      <c r="G34" s="68"/>
-      <c r="H34" s="68"/>
-      <c r="I34" s="68"/>
-      <c r="J34" s="68"/>
-      <c r="K34" s="68"/>
-      <c r="L34" s="68"/>
-      <c r="M34" s="68"/>
-      <c r="N34" s="68"/>
-      <c r="O34" s="68"/>
-      <c r="P34" s="68"/>
-      <c r="Q34" s="68"/>
-      <c r="R34" s="68"/>
-      <c r="S34" s="68"/>
-      <c r="T34" s="69"/>
+      <c r="B34" s="61" t="s">
+        <v>22</v>
+      </c>
+      <c r="C34" s="62"/>
+      <c r="D34" s="62"/>
+      <c r="E34" s="62"/>
+      <c r="F34" s="62"/>
+      <c r="G34" s="62"/>
+      <c r="H34" s="62"/>
+      <c r="I34" s="62"/>
+      <c r="J34" s="62"/>
+      <c r="K34" s="62"/>
+      <c r="L34" s="62"/>
+      <c r="M34" s="62"/>
+      <c r="N34" s="62"/>
+      <c r="O34" s="62"/>
+      <c r="P34" s="62"/>
+      <c r="Q34" s="62"/>
+      <c r="R34" s="62"/>
+      <c r="S34" s="62"/>
+      <c r="T34" s="63"/>
     </row>
     <row r="35" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B35" s="61" t="s">
-        <v>22</v>
-      </c>
-      <c r="C35" s="62"/>
-      <c r="D35" s="62"/>
-      <c r="E35" s="62"/>
-      <c r="F35" s="62"/>
-      <c r="G35" s="62"/>
-      <c r="H35" s="62"/>
-      <c r="I35" s="62"/>
-      <c r="J35" s="62"/>
-      <c r="K35" s="62"/>
-      <c r="L35" s="62"/>
-      <c r="M35" s="62"/>
-      <c r="N35" s="62"/>
-      <c r="O35" s="62"/>
-      <c r="P35" s="62"/>
-      <c r="Q35" s="62"/>
-      <c r="R35" s="62"/>
-      <c r="S35" s="62"/>
-      <c r="T35" s="63"/>
+      <c r="B35" s="64"/>
+      <c r="C35" s="65"/>
+      <c r="D35" s="65"/>
+      <c r="E35" s="65"/>
+      <c r="F35" s="65"/>
+      <c r="G35" s="65"/>
+      <c r="H35" s="65"/>
+      <c r="I35" s="65"/>
+      <c r="J35" s="65"/>
+      <c r="K35" s="65"/>
+      <c r="L35" s="65"/>
+      <c r="M35" s="65"/>
+      <c r="N35" s="65"/>
+      <c r="O35" s="65"/>
+      <c r="P35" s="65"/>
+      <c r="Q35" s="65"/>
+      <c r="R35" s="65"/>
+      <c r="S35" s="65"/>
+      <c r="T35" s="66"/>
     </row>
     <row r="36" spans="2:20" x14ac:dyDescent="0.4">
       <c r="B36" s="64"/>
@@ -2242,69 +2219,69 @@
       <c r="T37" s="66"/>
     </row>
     <row r="38" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B38" s="64"/>
-      <c r="C38" s="65"/>
-      <c r="D38" s="65"/>
-      <c r="E38" s="65"/>
-      <c r="F38" s="65"/>
-      <c r="G38" s="65"/>
-      <c r="H38" s="65"/>
-      <c r="I38" s="65"/>
-      <c r="J38" s="65"/>
-      <c r="K38" s="65"/>
-      <c r="L38" s="65"/>
-      <c r="M38" s="65"/>
-      <c r="N38" s="65"/>
-      <c r="O38" s="65"/>
-      <c r="P38" s="65"/>
-      <c r="Q38" s="65"/>
-      <c r="R38" s="65"/>
-      <c r="S38" s="65"/>
-      <c r="T38" s="66"/>
+      <c r="B38" s="67"/>
+      <c r="C38" s="68"/>
+      <c r="D38" s="68"/>
+      <c r="E38" s="68"/>
+      <c r="F38" s="68"/>
+      <c r="G38" s="68"/>
+      <c r="H38" s="68"/>
+      <c r="I38" s="68"/>
+      <c r="J38" s="68"/>
+      <c r="K38" s="68"/>
+      <c r="L38" s="68"/>
+      <c r="M38" s="68"/>
+      <c r="N38" s="68"/>
+      <c r="O38" s="68"/>
+      <c r="P38" s="68"/>
+      <c r="Q38" s="68"/>
+      <c r="R38" s="68"/>
+      <c r="S38" s="68"/>
+      <c r="T38" s="69"/>
     </row>
     <row r="39" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B39" s="67"/>
-      <c r="C39" s="68"/>
-      <c r="D39" s="68"/>
-      <c r="E39" s="68"/>
-      <c r="F39" s="68"/>
-      <c r="G39" s="68"/>
-      <c r="H39" s="68"/>
-      <c r="I39" s="68"/>
-      <c r="J39" s="68"/>
-      <c r="K39" s="68"/>
-      <c r="L39" s="68"/>
-      <c r="M39" s="68"/>
-      <c r="N39" s="68"/>
-      <c r="O39" s="68"/>
-      <c r="P39" s="68"/>
-      <c r="Q39" s="68"/>
-      <c r="R39" s="68"/>
-      <c r="S39" s="68"/>
-      <c r="T39" s="69"/>
+      <c r="B39" s="61" t="s">
+        <v>23</v>
+      </c>
+      <c r="C39" s="62"/>
+      <c r="D39" s="62"/>
+      <c r="E39" s="62"/>
+      <c r="F39" s="62"/>
+      <c r="G39" s="62"/>
+      <c r="H39" s="62"/>
+      <c r="I39" s="62"/>
+      <c r="J39" s="62"/>
+      <c r="K39" s="62"/>
+      <c r="L39" s="62"/>
+      <c r="M39" s="62"/>
+      <c r="N39" s="62"/>
+      <c r="O39" s="62"/>
+      <c r="P39" s="62"/>
+      <c r="Q39" s="62"/>
+      <c r="R39" s="62"/>
+      <c r="S39" s="62"/>
+      <c r="T39" s="63"/>
     </row>
     <row r="40" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B40" s="61" t="s">
-        <v>23</v>
-      </c>
-      <c r="C40" s="62"/>
-      <c r="D40" s="62"/>
-      <c r="E40" s="62"/>
-      <c r="F40" s="62"/>
-      <c r="G40" s="62"/>
-      <c r="H40" s="62"/>
-      <c r="I40" s="62"/>
-      <c r="J40" s="62"/>
-      <c r="K40" s="62"/>
-      <c r="L40" s="62"/>
-      <c r="M40" s="62"/>
-      <c r="N40" s="62"/>
-      <c r="O40" s="62"/>
-      <c r="P40" s="62"/>
-      <c r="Q40" s="62"/>
-      <c r="R40" s="62"/>
-      <c r="S40" s="62"/>
-      <c r="T40" s="63"/>
+      <c r="B40" s="64"/>
+      <c r="C40" s="65"/>
+      <c r="D40" s="65"/>
+      <c r="E40" s="65"/>
+      <c r="F40" s="65"/>
+      <c r="G40" s="65"/>
+      <c r="H40" s="65"/>
+      <c r="I40" s="65"/>
+      <c r="J40" s="65"/>
+      <c r="K40" s="65"/>
+      <c r="L40" s="65"/>
+      <c r="M40" s="65"/>
+      <c r="N40" s="65"/>
+      <c r="O40" s="65"/>
+      <c r="P40" s="65"/>
+      <c r="Q40" s="65"/>
+      <c r="R40" s="65"/>
+      <c r="S40" s="65"/>
+      <c r="T40" s="66"/>
     </row>
     <row r="41" spans="2:20" x14ac:dyDescent="0.4">
       <c r="B41" s="64"/>
@@ -2475,56 +2452,60 @@
       <c r="T48" s="66"/>
     </row>
     <row r="49" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B49" s="64"/>
-      <c r="C49" s="65"/>
-      <c r="D49" s="65"/>
-      <c r="E49" s="65"/>
-      <c r="F49" s="65"/>
-      <c r="G49" s="65"/>
-      <c r="H49" s="65"/>
-      <c r="I49" s="65"/>
-      <c r="J49" s="65"/>
-      <c r="K49" s="65"/>
-      <c r="L49" s="65"/>
-      <c r="M49" s="65"/>
-      <c r="N49" s="65"/>
-      <c r="O49" s="65"/>
-      <c r="P49" s="65"/>
-      <c r="Q49" s="65"/>
-      <c r="R49" s="65"/>
-      <c r="S49" s="65"/>
-      <c r="T49" s="66"/>
-    </row>
-    <row r="50" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B50" s="67"/>
-      <c r="C50" s="68"/>
-      <c r="D50" s="68"/>
-      <c r="E50" s="68"/>
-      <c r="F50" s="68"/>
-      <c r="G50" s="68"/>
-      <c r="H50" s="68"/>
-      <c r="I50" s="68"/>
-      <c r="J50" s="68"/>
-      <c r="K50" s="68"/>
-      <c r="L50" s="68"/>
-      <c r="M50" s="68"/>
-      <c r="N50" s="68"/>
-      <c r="O50" s="68"/>
-      <c r="P50" s="68"/>
-      <c r="Q50" s="68"/>
-      <c r="R50" s="68"/>
-      <c r="S50" s="68"/>
-      <c r="T50" s="69"/>
-    </row>
-    <row r="52" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B52" s="31" t="s">
+      <c r="B49" s="67"/>
+      <c r="C49" s="68"/>
+      <c r="D49" s="68"/>
+      <c r="E49" s="68"/>
+      <c r="F49" s="68"/>
+      <c r="G49" s="68"/>
+      <c r="H49" s="68"/>
+      <c r="I49" s="68"/>
+      <c r="J49" s="68"/>
+      <c r="K49" s="68"/>
+      <c r="L49" s="68"/>
+      <c r="M49" s="68"/>
+      <c r="N49" s="68"/>
+      <c r="O49" s="68"/>
+      <c r="P49" s="68"/>
+      <c r="Q49" s="68"/>
+      <c r="R49" s="68"/>
+      <c r="S49" s="68"/>
+      <c r="T49" s="69"/>
+    </row>
+    <row r="51" spans="2:20" x14ac:dyDescent="0.4">
+      <c r="B51" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="C52" s="44"/>
-      <c r="D52" s="32"/>
-      <c r="E52" s="14" t="s">
-        <v>31</v>
-      </c>
+      <c r="C51" s="44"/>
+      <c r="D51" s="32"/>
+      <c r="E51" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="F51" s="14"/>
+      <c r="G51" s="14"/>
+      <c r="H51" s="4"/>
+      <c r="I51"/>
+      <c r="J51"/>
+      <c r="K51"/>
+      <c r="L51"/>
+      <c r="M51" s="4"/>
+      <c r="N51" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="O51" s="14"/>
+      <c r="P51" s="14"/>
+      <c r="Q51" s="14"/>
+      <c r="R51" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="S51" s="44"/>
+      <c r="T51" s="32"/>
+    </row>
+    <row r="52" spans="2:20" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B52" s="21"/>
+      <c r="C52" s="71"/>
+      <c r="D52" s="22"/>
+      <c r="E52" s="14"/>
       <c r="F52" s="14"/>
       <c r="G52" s="14"/>
       <c r="H52" s="4"/>
@@ -2533,22 +2514,18 @@
       <c r="K52"/>
       <c r="L52"/>
       <c r="M52" s="4"/>
-      <c r="N52" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="O52" s="14"/>
-      <c r="P52" s="14"/>
-      <c r="Q52" s="14"/>
-      <c r="R52" s="31" t="s">
-        <v>11</v>
-      </c>
-      <c r="S52" s="44"/>
-      <c r="T52" s="32"/>
+      <c r="N52" s="14"/>
+      <c r="O52" s="22"/>
+      <c r="P52" s="22"/>
+      <c r="Q52" s="48"/>
+      <c r="R52" s="14"/>
+      <c r="S52" s="22"/>
+      <c r="T52" s="48"/>
     </row>
     <row r="53" spans="2:20" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B53" s="21"/>
-      <c r="C53" s="71"/>
-      <c r="D53" s="22"/>
+      <c r="B53" s="23"/>
+      <c r="C53" s="72"/>
+      <c r="D53" s="24"/>
       <c r="E53" s="14"/>
       <c r="F53" s="14"/>
       <c r="G53" s="14"/>
@@ -2558,18 +2535,18 @@
       <c r="K53"/>
       <c r="L53"/>
       <c r="M53" s="4"/>
-      <c r="N53" s="14"/>
-      <c r="O53" s="22"/>
-      <c r="P53" s="22"/>
-      <c r="Q53" s="48"/>
-      <c r="R53" s="14"/>
-      <c r="S53" s="22"/>
-      <c r="T53" s="48"/>
-    </row>
-    <row r="54" spans="2:20" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B54" s="23"/>
-      <c r="C54" s="72"/>
-      <c r="D54" s="24"/>
+      <c r="N53" s="49"/>
+      <c r="O53" s="50"/>
+      <c r="P53" s="50"/>
+      <c r="Q53" s="51"/>
+      <c r="R53" s="49"/>
+      <c r="S53" s="50"/>
+      <c r="T53" s="51"/>
+    </row>
+    <row r="54" spans="2:20" x14ac:dyDescent="0.4">
+      <c r="B54" s="25"/>
+      <c r="C54" s="73"/>
+      <c r="D54" s="26"/>
       <c r="E54" s="14"/>
       <c r="F54" s="14"/>
       <c r="G54" s="14"/>
@@ -2578,27 +2555,6 @@
       <c r="J54"/>
       <c r="K54"/>
       <c r="L54"/>
-      <c r="M54" s="4"/>
-      <c r="N54" s="49"/>
-      <c r="O54" s="50"/>
-      <c r="P54" s="50"/>
-      <c r="Q54" s="51"/>
-      <c r="R54" s="49"/>
-      <c r="S54" s="50"/>
-      <c r="T54" s="51"/>
-    </row>
-    <row r="55" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B55" s="25"/>
-      <c r="C55" s="73"/>
-      <c r="D55" s="26"/>
-      <c r="E55" s="14"/>
-      <c r="F55" s="14"/>
-      <c r="G55" s="14"/>
-      <c r="H55" s="4"/>
-      <c r="I55"/>
-      <c r="J55"/>
-      <c r="K55"/>
-      <c r="L55"/>
     </row>
   </sheetData>
   <mergeCells count="75">
@@ -2607,30 +2563,30 @@
     <mergeCell ref="P2:Q2"/>
     <mergeCell ref="N3:O3"/>
     <mergeCell ref="N2:O2"/>
-    <mergeCell ref="N53:Q54"/>
-    <mergeCell ref="R53:T54"/>
+    <mergeCell ref="N52:Q53"/>
+    <mergeCell ref="R52:T53"/>
     <mergeCell ref="H5:J5"/>
     <mergeCell ref="B15:B18"/>
-    <mergeCell ref="N25:O25"/>
+    <mergeCell ref="N22:O22"/>
     <mergeCell ref="H6:J8"/>
-    <mergeCell ref="C20:R20"/>
-    <mergeCell ref="C25:I25"/>
+    <mergeCell ref="C22:I22"/>
+    <mergeCell ref="S25:T25"/>
+    <mergeCell ref="C25:R25"/>
+    <mergeCell ref="B52:D54"/>
+    <mergeCell ref="B51:D51"/>
     <mergeCell ref="S19:T19"/>
-    <mergeCell ref="C19:R19"/>
-    <mergeCell ref="B53:D55"/>
-    <mergeCell ref="B52:D52"/>
-    <mergeCell ref="S22:T22"/>
-    <mergeCell ref="N52:Q52"/>
-    <mergeCell ref="R52:T52"/>
-    <mergeCell ref="C28:R28"/>
-    <mergeCell ref="C26:R26"/>
-    <mergeCell ref="B40:T50"/>
-    <mergeCell ref="B35:T39"/>
-    <mergeCell ref="B30:T34"/>
-    <mergeCell ref="S26:T26"/>
-    <mergeCell ref="S28:T28"/>
-    <mergeCell ref="E52:G52"/>
-    <mergeCell ref="E53:G55"/>
+    <mergeCell ref="N51:Q51"/>
+    <mergeCell ref="R51:T51"/>
+    <mergeCell ref="C27:R27"/>
+    <mergeCell ref="S23:T23"/>
+    <mergeCell ref="C24:R24"/>
+    <mergeCell ref="B39:T49"/>
+    <mergeCell ref="B34:T38"/>
+    <mergeCell ref="B29:T33"/>
+    <mergeCell ref="S24:T24"/>
+    <mergeCell ref="S27:T27"/>
+    <mergeCell ref="E51:G51"/>
+    <mergeCell ref="E52:G54"/>
     <mergeCell ref="S14:T14"/>
     <mergeCell ref="C15:R15"/>
     <mergeCell ref="S10:T10"/>
@@ -2643,18 +2599,18 @@
     <mergeCell ref="S12:T12"/>
     <mergeCell ref="S15:T18"/>
     <mergeCell ref="C11:R11"/>
-    <mergeCell ref="C22:R22"/>
-    <mergeCell ref="C21:R21"/>
+    <mergeCell ref="C19:R19"/>
+    <mergeCell ref="C23:R23"/>
     <mergeCell ref="B2:C2"/>
-    <mergeCell ref="C27:R27"/>
-    <mergeCell ref="S27:T27"/>
+    <mergeCell ref="C26:R26"/>
+    <mergeCell ref="S26:T26"/>
     <mergeCell ref="D2:K2"/>
     <mergeCell ref="E6:G8"/>
     <mergeCell ref="E5:G5"/>
     <mergeCell ref="D3:K3"/>
     <mergeCell ref="R3:T3"/>
     <mergeCell ref="R2:T2"/>
-    <mergeCell ref="C24:R24"/>
+    <mergeCell ref="C21:R21"/>
     <mergeCell ref="R6:T7"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B6:D8"/>
@@ -2662,9 +2618,9 @@
     <mergeCell ref="N6:Q7"/>
     <mergeCell ref="N5:Q5"/>
     <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B23:B25"/>
-    <mergeCell ref="C23:R23"/>
-    <mergeCell ref="S23:T25"/>
+    <mergeCell ref="B20:B22"/>
+    <mergeCell ref="C20:R20"/>
+    <mergeCell ref="S20:T22"/>
     <mergeCell ref="K16:O16"/>
     <mergeCell ref="C16:J16"/>
     <mergeCell ref="P16:Q16"/>
@@ -2681,12 +2637,12 @@
   <phoneticPr fontId="1"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="3.937007874015748E-2" right="3.937007874015748E-2" top="0.55118110236220474" bottom="0.55118110236220474" header="0.11811023622047245" footer="0.11811023622047245"/>
-  <pageSetup paperSize="9" scale="71" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="73" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddFooter>&amp;LGxC-A-PR21-F01&amp;R版: 01</oddFooter>
   </headerFooter>
   <rowBreaks count="1" manualBreakCount="1">
-    <brk id="22" max="16383" man="1"/>
+    <brk id="19" max="16383" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
</xml_diff>